<commit_message>
3.5.6: export menu bug, weight bug, add circular progress on save
</commit_message>
<xml_diff>
--- a/results/SamChigome/analysis/Analysis_v2.xlsx
+++ b/results/SamChigome/analysis/Analysis_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owuor\owProjects\StructuralGT\results\SamChigome\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/owuorjnr/owProjects/StructuralGT/results/SamChigome/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78CFBDA-658D-470D-8EF2-509AD72E95B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAE551D-CCC8-0D49-A389-38BB5081E879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12825" yWindow="0" windowWidth="17445" windowHeight="14775" firstSheet="5" activeTab="7" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16760" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
   </bookViews>
   <sheets>
     <sheet name="SGT Descriptors" sheetId="2" r:id="rId1"/>
@@ -44,9 +44,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="34">
-  <si>
-    <t>ND</t>
-  </si>
   <si>
     <t>CC</t>
   </si>
@@ -82,9 +79,6 @@
   </si>
   <si>
     <t>ANC: Average Node Connectivity</t>
-  </si>
-  <si>
-    <t>ND: Average Node Degree</t>
   </si>
   <si>
     <t>CC: Avg. Closessness Centrality</t>
@@ -145,6 +139,12 @@
   </si>
   <si>
     <t>log-y-fit</t>
+  </si>
+  <si>
+    <t>AD: Average Node Degree</t>
+  </si>
+  <si>
+    <t>AD</t>
   </si>
 </sst>
 </file>
@@ -610,7 +610,7 @@
                   <c:v>Edges</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>ND</c:v>
+                  <c:v>AD</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Diameter</c:v>
@@ -719,7 +719,7 @@
                   <c:v>Edges</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>ND</c:v>
+                  <c:v>AD</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Diameter</c:v>
@@ -828,7 +828,7 @@
                   <c:v>Edges</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>ND</c:v>
+                  <c:v>AD</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Diameter</c:v>
@@ -943,7 +943,7 @@
                   <c:v>Edges</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>ND</c:v>
+                  <c:v>AD</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Diameter</c:v>
@@ -1162,6 +1162,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1169,7 +1170,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1780,6 +1780,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1787,7 +1788,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2589,6 +2589,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2596,7 +2597,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5136,45 +5136,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C9C1606-6F01-4D2D-8971-65E27527CE3F}">
   <dimension ref="A2:T34"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="23"/>
-    <col min="8" max="8" width="8.85546875" style="8"/>
+    <col min="2" max="2" width="13.1640625" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" style="23"/>
+    <col min="8" max="8" width="8.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C2" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="F2" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="19" t="s">
-        <v>23</v>
-      </c>
       <c r="H2" s="24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>9</v>
       </c>
       <c r="C3">
         <v>7785</v>
@@ -5197,15 +5197,15 @@
         <v>11.195237082497776</v>
       </c>
       <c r="O3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>13854</v>
@@ -5228,15 +5228,15 @@
         <v>34.346275877694026</v>
       </c>
       <c r="O4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>3.5591499999999998</v>
@@ -5259,15 +5259,15 @@
         <v>4.8312964098675797E-3</v>
       </c>
       <c r="O5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>111</v>
@@ -5292,7 +5292,7 @@
       <c r="I6" s="2"/>
       <c r="N6" s="1"/>
       <c r="O6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -5300,12 +5300,12 @@
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7">
         <v>4.6000000000000001E-4</v>
@@ -5328,15 +5328,15 @@
         <v>0</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8">
         <v>5.1799999999999997E-3</v>
@@ -5359,15 +5359,15 @@
         <v>1.499999999999987E-5</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9">
         <v>1.3500000000000001E-3</v>
@@ -5390,12 +5390,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10">
         <v>2.4809999999999999E-2</v>
@@ -5418,12 +5418,12 @@
         <v>2.645751311064636E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>7329</v>
@@ -5446,12 +5446,12 @@
         <v>19.510680835549195</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12">
         <v>12000</v>
@@ -5474,12 +5474,12 @@
         <v>36.514837167011073</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C13">
         <v>3.2746599999999999</v>
@@ -5502,12 +5502,12 @@
         <v>7.4972528302039761E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C14">
         <v>116</v>
@@ -5530,12 +5530,12 @@
         <v>2.0615528128088303</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>4.4999999999999999E-4</v>
@@ -5558,12 +5558,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16">
         <v>5.8900000000000003E-3</v>
@@ -5586,12 +5586,12 @@
         <v>2.0615528128088444E-5</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C17">
         <v>8.0999999999999996E-4</v>
@@ -5614,12 +5614,12 @@
         <v>6.9282032302755148E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18">
         <v>2.3220000000000001E-2</v>
@@ -5642,12 +5642,12 @@
         <v>1.0812801055539042E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19">
         <v>7769</v>
@@ -5670,12 +5670,12 @@
         <v>9.1469484893414954</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C20">
         <v>13781</v>
@@ -5698,12 +5698,12 @@
         <v>34.837719022155667</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C21">
         <v>3.5476899999999998</v>
@@ -5726,12 +5726,12 @@
         <v>4.855066082626063E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C22">
         <v>114</v>
@@ -5754,12 +5754,12 @@
         <v>0.9574271077563381</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23">
         <v>4.6000000000000001E-4</v>
@@ -5782,12 +5782,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24">
         <v>5.2900000000000004E-3</v>
@@ -5810,12 +5810,12 @@
         <v>9.5742710775634437E-6</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C25">
         <v>1.2700000000000001E-3</v>
@@ -5838,12 +5838,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26">
         <v>2.4379999999999999E-2</v>
@@ -5866,12 +5866,12 @@
         <v>4.3969686527575916E-5</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" s="22">
         <v>7433</v>
@@ -5894,12 +5894,12 @@
         <v>18.357559750685819</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C28" s="22">
         <v>13923</v>
@@ -5922,12 +5922,12 @@
         <v>26.901053263146903</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C29" s="22">
         <v>3.74627</v>
@@ -5950,12 +5950,12 @@
         <v>4.2697335982470538E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C30" s="22">
         <v>98</v>
@@ -5978,12 +5978,12 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" s="22">
         <v>5.0000000000000001E-4</v>
@@ -6006,12 +6006,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="22">
         <v>4.9399999999999999E-3</v>
@@ -6034,12 +6034,12 @@
         <v>1.8257418583505586E-5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C33" s="22">
         <v>9.1E-4</v>
@@ -6062,12 +6062,12 @@
         <v>5.0000000000000131E-6</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C34" s="22">
         <v>2.7210000000000002E-2</v>
@@ -6101,51 +6101,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62EDEAF-E711-4AB0-9613-3030E8997E92}">
   <dimension ref="A2:K46"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.140625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.1640625" style="21" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
     <col min="4" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" customWidth="1"/>
+    <col min="7" max="7" width="13.5" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="E2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="F2" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="G2" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="H2" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="I2" s="25" t="s">
         <v>31</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="25" t="s">
-        <v>33</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -6172,9 +6172,9 @@
         <v>1.9407258214499949</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -6201,9 +6201,9 @@
         <v>2.562815299227351</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -6230,9 +6230,9 @@
         <v>2.9121547178957279</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -6259,9 +6259,9 @@
         <v>3.172274295925777</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -6288,9 +6288,9 @@
         <v>3.3698888174679968</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -6317,9 +6317,9 @@
         <v>3.5346957486974269</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -6346,9 +6346,9 @@
         <v>3.6729515048586889</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -6375,9 +6375,9 @@
         <v>3.7898343812554618</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -6404,9 +6404,9 @@
         <v>3.897398635328154</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -6433,9 +6433,9 @@
         <v>3.9931722148676481</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -6462,9 +6462,9 @@
         <v>4.1944951179246281</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -6491,9 +6491,9 @@
         <v>1.86397049175859</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -6520,9 +6520,9 @@
         <v>2.4779284189133</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -6549,9 +6549,9 @@
         <v>2.852938154437608</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -6578,9 +6578,9 @@
         <v>3.109166756016247</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -6607,9 +6607,9 @@
         <v>3.3113664252333779</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -6636,9 +6636,9 @@
         <v>3.4712043182454062</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -6665,9 +6665,9 @@
         <v>3.6082399976904238</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -6694,9 +6694,9 @@
         <v>3.731804427834386</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -6723,9 +6723,9 @@
         <v>3.833695311408003</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -6752,9 +6752,9 @@
         <v>3.926075920414569</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -6781,9 +6781,9 @@
         <v>4.1334298429872316</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -6810,9 +6810,9 @@
         <v>1.9457851526211629</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -6839,9 +6839,9 @@
         <v>2.5428575354672329</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -6868,9 +6868,9 @@
         <v>2.9060938385819308</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -6897,9 +6897,9 @@
         <v>3.173286583552831</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -6926,9 +6926,9 @@
         <v>3.3675632548424721</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -6955,9 +6955,9 @@
         <v>3.5325845762341381</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -6984,9 +6984,9 @@
         <v>3.6678075935634209</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -7013,9 +7013,9 @@
         <v>3.7878260508153412</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -7042,9 +7042,9 @@
         <v>3.8928997078867922</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -7071,9 +7071,9 @@
         <v>3.9863333020807432</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -7100,9 +7100,9 @@
         <v>4.1922519336383131</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -7129,9 +7129,9 @@
         <v>1.9260214176428361</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -7158,9 +7158,9 @@
         <v>2.571653336874856</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -7187,9 +7187,9 @@
         <v>2.9223498383860051</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -7216,9 +7216,9 @@
         <v>3.1777018852706291</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -7245,9 +7245,9 @@
         <v>3.3755861225721402</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -7274,9 +7274,9 @@
         <v>3.535610544036119</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -7303,9 +7303,9 @@
         <v>3.6671525688381741</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -7332,9 +7332,9 @@
         <v>3.786746806642395</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -7361,9 +7361,9 @@
         <v>3.890916954426618</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -7390,9 +7390,9 @@
         <v>3.9887603913317902</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -7429,45 +7429,45 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1057D40A-C89C-420E-9857-286802B3D7FB}">
   <dimension ref="A2:K46"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
       </c>
       <c r="J2" s="30"/>
       <c r="K2" s="30"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -7494,9 +7494,9 @@
         <v>0.51006056698685842</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -7523,9 +7523,9 @@
         <v>0.52392876133226562</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -7552,9 +7552,9 @@
         <v>0.53171655894606573</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -7581,9 +7581,9 @@
         <v>0.53751538530470266</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -7610,9 +7610,9 @@
         <v>0.5419207910994025</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -7639,9 +7639,9 @@
         <v>0.54559481972937696</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -7668,9 +7668,9 @@
         <v>0.5486769449931993</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -7697,9 +7697,9 @@
         <v>0.55128260624198311</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -7726,9 +7726,9 @@
         <v>0.5536805281380881</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -7755,9 +7755,9 @@
         <v>0.55581560140593145</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -7784,9 +7784,9 @@
         <v>0.56030367787324464</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -7813,9 +7813,9 @@
         <v>0.46919556731156259</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -7842,9 +7842,9 @@
         <v>0.48371554040580361</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -7871,9 +7871,9 @@
         <v>0.49258444009592722</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -7900,9 +7900,9 @@
         <v>0.49864419148335293</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -7929,9 +7929,9 @@
         <v>0.50342617022626657</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -7958,9 +7958,9 @@
         <v>0.50720630206157058</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -7987,9 +7987,9 @@
         <v>0.51044716644410881</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -8016,9 +8016,9 @@
         <v>0.51336943867440676</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -8045,9 +8045,9 @@
         <v>0.51577913618396354</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -8074,9 +8074,9 @@
         <v>0.51796391774289097</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -8103,9 +8103,9 @@
         <v>0.52286779347048906</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -8132,9 +8132,9 @@
         <v>0.5027907425585495</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -8161,9 +8161,9 @@
         <v>0.51752351891033554</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -8190,9 +8190,9 @@
         <v>0.52648638400071113</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -8219,9 +8219,9 @@
         <v>0.5330793718319552</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -8248,9 +8248,9 @@
         <v>0.53787315367601962</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -8277,9 +8277,9 @@
         <v>0.54194505901143419</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -8306,9 +8306,9 @@
         <v>0.54528169043027441</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -8335,9 +8335,9 @@
         <v>0.54824314893945958</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -8364,9 +8364,9 @@
         <v>0.55083584412110398</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -8393,9 +8393,9 @@
         <v>0.55314132045287046</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -8422,9 +8422,9 @@
         <v>0.55822236796497027</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -8451,9 +8451,9 @@
         <v>0.5295421413759962</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -8480,9 +8480,9 @@
         <v>0.54329225422603167</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -8509,9 +8509,9 @@
         <v>0.55076108643251065</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -8538,9 +8538,9 @@
         <v>0.55619935451771862</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -8567,9 +8567,9 @@
         <v>0.56041372266323342</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -8596,9 +8596,9 @@
         <v>0.56382178504111069</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -8625,9 +8625,9 @@
         <v>0.56662325385278578</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -8654,9 +8654,9 @@
         <v>0.5691702689817435</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -8683,9 +8683,9 @@
         <v>0.57138879511865093</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -8712,9 +8712,9 @@
         <v>0.57347258041334603</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -8750,12 +8750,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5B1F077-EC4F-492C-BDC7-962283AFF80E}">
   <dimension ref="A1:K46"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -8766,40 +8766,40 @@
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -8826,9 +8826,9 @@
         <v>1.019491982774134</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -8855,9 +8855,9 @@
         <v>1.3033313549351371</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -8884,9 +8884,9 @@
         <v>1.462723668754998</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -8913,9 +8913,9 @@
         <v>1.581407845794331</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -8942,9 +8942,9 @@
         <v>1.671572980759876</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -8971,9 +8971,9 @@
         <v>1.746769070002661</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -9000,9 +9000,9 @@
         <v>1.809850714088115</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -9029,9 +9029,9 @@
         <v>1.8631806022118711</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -9058,9 +9058,9 @@
         <v>1.9122587034072851</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -9087,9 +9087,9 @@
         <v>1.955957099951827</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -9116,9 +9116,9 @@
         <v>2.0478142498420469</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -9145,9 +9145,9 @@
         <v>1.0567165444598361</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -9174,9 +9174,9 @@
         <v>1.332620838320542</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -9203,9 +9203,9 @@
         <v>1.50114508354077</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -9232,9 +9232,9 @@
         <v>1.6162907120255969</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -9261,9 +9261,9 @@
         <v>1.707156477392876</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -9290,9 +9290,9 @@
         <v>1.7789854400190941</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -9319,9 +9319,9 @@
         <v>1.840567399789885</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -9348,9 +9348,9 @@
         <v>1.8960955644039721</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -9377,9 +9377,9 @@
         <v>1.941883933671396</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -9406,9 +9406,9 @@
         <v>1.9833985156436491</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -9435,9 +9435,9 @@
         <v>2.0765805319615871</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -9464,9 +9464,9 @@
         <v>1.032507679674538</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -9493,9 +9493,9 @@
         <v>1.305591312664973</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -9522,9 +9522,9 @@
         <v>1.4717250882982511</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -9551,9 +9551,9 @@
         <v>1.593931319237174</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -9580,9 +9580,9 @@
         <v>1.682787847734057</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -9609,9 +9609,9 @@
         <v>1.758263825624222</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -9638,9 +9638,9 @@
         <v>1.820110921382007</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -9667,9 +9667,9 @@
         <v>1.875003891269563</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -9696,9 +9696,9 @@
         <v>1.923061541948176</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -9725,9 +9725,9 @@
         <v>1.9657953646452071</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -9754,9 +9754,9 @@
         <v>2.059976588935156</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -9783,9 +9783,9 @@
         <v>0.97075157678277413</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -9812,9 +9812,9 @@
         <v>1.2661612437056791</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -9841,9 +9841,9 @@
         <v>1.426622852892641</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -9870,9 +9870,9 @@
         <v>1.5434594913413671</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -9899,9 +9899,9 @@
         <v>1.6340016638846131</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -9928,9 +9928,9 @@
         <v>1.7072210318186449</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -9957,9 +9957,9 @@
         <v>1.7674082446493891</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -9986,9 +9986,9 @@
         <v>1.822128733062768</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -10015,9 +10015,9 @@
         <v>1.869791910398938</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -10044,9 +10044,9 @@
         <v>1.9145602935066539</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -10081,16 +10081,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E56A98-F0FD-4ECE-85FB-F0A28ED9F179}">
   <dimension ref="A1:U46"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -10101,39 +10101,39 @@
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
-      </c>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -10160,9 +10160,9 @@
         <v>-1.21265489211005</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -10189,9 +10189,9 @@
         <v>-1.810313726683723</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -10218,9 +10218,9 @@
         <v>-2.1459339184573412</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -10247,9 +10247,9 @@
         <v>-2.3958381033194329</v>
       </c>
     </row>
-    <row r="7" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -10276,9 +10276,9 @@
         <v>-2.5856919247692578</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -10305,9 +10305,9 @@
         <v>-2.744026572704739</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -10334,9 +10334,9 @@
         <v>-2.8768527609818122</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -10364,9 +10364,9 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -10403,9 +10403,9 @@
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -10432,9 +10432,9 @@
         <v>-3.184497791458929</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -10461,9 +10461,9 @@
         <v>-3.3779143591911449</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -10491,9 +10491,9 @@
       </c>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -10520,9 +10520,9 @@
         <v>-1.8039271867889879</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -10559,9 +10559,9 @@
       <c r="T16" s="5"/>
       <c r="U16" s="2"/>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -10589,9 +10589,9 @@
       </c>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -10618,9 +10618,9 @@
         <v>-2.603543062578344</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -10647,9 +10647,9 @@
         <v>-2.7568945006408572</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -10676,9 +10676,9 @@
         <v>-2.8883690722381301</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -10714,9 +10714,9 @@
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -10743,9 +10743,9 @@
         <v>-3.104675080318605</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -10772,9 +10772,9 @@
         <v>-3.1933067494008651</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -10801,9 +10801,9 @@
         <v>-3.3922459472044051</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -10830,9 +10830,9 @@
         <v>-1.231432449729323</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -10867,9 +10867,9 @@
       <c r="S26" s="19"/>
       <c r="T26" s="19"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -10905,9 +10905,9 @@
       <c r="T27" s="5"/>
       <c r="U27" s="2"/>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -10934,9 +10934,9 @@
         <v>-2.4052530332983642</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -10963,9 +10963,9 @@
         <v>-2.59103363600933</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -10992,9 +10992,9 @@
         <v>-2.7488382779397891</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -11021,9 +11021,9 @@
         <v>-2.8781477492883911</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -11050,9 +11050,9 @@
         <v>-2.9929175833435551</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -11079,9 +11079,9 @@
         <v>-3.093396180234258</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -11108,9 +11108,9 @@
         <v>-3.1827437551519129</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -11137,9 +11137,9 @@
         <v>-3.379657194250056</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -11166,9 +11166,9 @@
         <v>-1.159694323071728</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -11195,9 +11195,9 @@
         <v>-1.7808596489171771</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -11224,9 +11224,9 @@
         <v>-2.118266304544044</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -11253,9 +11253,9 @@
         <v>-2.363941638559536</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -11282,9 +11282,9 @@
         <v>-2.5543269387306968</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -11311,9 +11311,9 @@
         <v>-2.708287142588246</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -11340,9 +11340,9 @@
         <v>-2.8348443066078501</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -11369,9 +11369,9 @@
         <v>-2.9499064518984079</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -11398,9 +11398,9 @@
         <v>-3.0501290119427198</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -11427,9 +11427,9 @@
         <v>-3.1442646154601759</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -11466,20 +11466,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{908D8F90-1399-4559-8642-02E0AC650D8E}">
   <dimension ref="A1:AC46"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" style="6" customWidth="1"/>
-    <col min="4" max="5" width="10.42578125" style="6" customWidth="1"/>
-    <col min="6" max="13" width="9.42578125" style="7" customWidth="1"/>
-    <col min="14" max="17" width="9.140625" style="8"/>
-    <col min="18" max="21" width="9.140625" style="9"/>
-    <col min="22" max="25" width="9.42578125" style="7" customWidth="1"/>
-    <col min="26" max="29" width="9.140625" style="10"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="6" customWidth="1"/>
+    <col min="4" max="5" width="10.5" style="6" customWidth="1"/>
+    <col min="6" max="13" width="9.5" style="7" customWidth="1"/>
+    <col min="14" max="17" width="9.1640625" style="8"/>
+    <col min="18" max="21" width="9.1640625" style="9"/>
+    <col min="22" max="25" width="9.5" style="7" customWidth="1"/>
+    <col min="26" max="29" width="9.1640625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -11490,33 +11490,33 @@
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
       </c>
       <c r="J2" s="14"/>
       <c r="K2" s="14"/>
@@ -11527,9 +11527,9 @@
       <c r="X2" s="16"/>
       <c r="Y2" s="16"/>
     </row>
-    <row r="3" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -11576,9 +11576,9 @@
       <c r="AB3" s="13"/>
       <c r="AC3" s="13"/>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -11613,9 +11613,9 @@
       <c r="X4" s="16"/>
       <c r="Y4" s="16"/>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -11650,9 +11650,9 @@
       <c r="X5" s="16"/>
       <c r="Y5" s="16"/>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -11687,9 +11687,9 @@
       <c r="X6" s="16"/>
       <c r="Y6" s="16"/>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -11724,9 +11724,9 @@
       <c r="X7" s="16"/>
       <c r="Y7" s="16"/>
     </row>
-    <row r="8" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -11773,9 +11773,9 @@
       <c r="AB8" s="13"/>
       <c r="AC8" s="13"/>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -11802,9 +11802,9 @@
         <v>-2.0505368001804869</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -11831,9 +11831,9 @@
         <v>-2.1107997594094758</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -11860,9 +11860,9 @@
         <v>-2.1662581846083468</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -11889,9 +11889,9 @@
         <v>-2.2156375248241922</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -11918,9 +11918,9 @@
         <v>-2.3194364239683218</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -11947,9 +11947,9 @@
         <v>-1.075552118201571</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -11976,9 +11976,9 @@
         <v>-1.3981531755619481</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -12005,9 +12005,9 @@
         <v>-1.5952001259307329</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -12034,9 +12034,9 @@
         <v>-1.7298341360791349</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -12063,9 +12063,9 @@
         <v>-1.8360789196421761</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -12092,9 +12092,9 @@
         <v>-1.92006492423845</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -12121,9 +12121,9 @@
         <v>-1.992069622166099</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -12150,9 +12150,9 @@
         <v>-2.056995920945738</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -12179,9 +12179,9 @@
         <v>-2.1105339653660828</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -12208,9 +12208,9 @@
         <v>-2.1590748845838328</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -12237,9 +12237,9 @@
         <v>-2.2680279442499329</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -12266,9 +12266,9 @@
         <v>-1.15188756303448</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -12295,9 +12295,9 @@
         <v>-1.460781329376569</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -12324,9 +12324,9 @@
         <v>-1.648700638600761</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -12353,9 +12353,9 @@
         <v>-1.7869320753654721</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -12382,9 +12382,9 @@
         <v>-1.887440580583897</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -12411,9 +12411,9 @@
         <v>-1.972813910444577</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -12440,9 +12440,9 @@
         <v>-2.0427711690936552</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -12469,9 +12469,9 @@
         <v>-2.1048623901184769</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -12498,9 +12498,9 @@
         <v>-2.1592219595921591</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -12527,9 +12527,9 @@
         <v>-2.2075595743313889</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -12556,9 +12556,9 @@
         <v>-2.3140910158940202</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -12585,9 +12585,9 @@
         <v>-1.172239015000931</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -12614,9 +12614,9 @@
         <v>-1.5042845632925339</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -12643,9 +12643,9 @@
         <v>-1.68464617284048</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -12672,9 +12672,9 @@
         <v>-1.815972564689327</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -12701,9 +12701,9 @@
         <v>-1.9177435244510499</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -12730,9 +12730,9 @@
         <v>-2.0000433537845481</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -12759,9 +12759,9 @@
         <v>-2.0676948165572382</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -12788,9 +12788,9 @@
         <v>-2.1292015870270982</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -12817,9 +12817,9 @@
         <v>-2.1827758184216259</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -12846,9 +12846,9 @@
         <v>-2.233096251296999</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -12883,9 +12883,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{706895DB-66F3-AF47-A56B-9367486E6A96}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -12896,38 +12896,38 @@
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -12954,9 +12954,9 @@
         <v>-0.96566965972394891</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -12983,9 +12983,9 @@
         <v>-1.4890379727906491</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -13012,9 +13012,9 @@
         <v>-1.782939716458471</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -13041,9 +13041,9 @@
         <v>-2.0017801720720469</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -13070,9 +13070,9 @@
         <v>-2.168034678009938</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -13099,9 +13099,9 @@
         <v>-2.306687924304061</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -13128,9 +13128,9 @@
         <v>-2.4230034777071001</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -13157,9 +13157,9 @@
         <v>-2.521337874978574</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -13186,9 +13186,9 @@
         <v>-2.6118324488483009</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -13215,9 +13215,9 @@
         <v>-2.6924074441673569</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -13244,9 +13244,9 @@
         <v>-2.8617818379138669</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -13273,9 +13273,9 @@
         <v>-0.95719864308073777</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -13302,9 +13302,9 @@
         <v>-1.513406240369789</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -13331,9 +13331,9 @@
         <v>-1.8531416761880439</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -13360,9 +13360,9 @@
         <v>-2.085268811513517</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -13389,9 +13389,9 @@
         <v>-2.268449103213801</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -13418,9 +13418,9 @@
         <v>-2.413252267235106</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -13447,9 +13447,9 @@
         <v>-2.537398047647482</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -13476,9 +13476,9 @@
         <v>-2.649339716222836</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -13505,9 +13505,9 @@
         <v>-2.7416465031076962</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -13534,9 +13534,9 @@
         <v>-2.8253375742691471</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -13563,9 +13563,9 @@
         <v>-3.0131872981046008</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -13592,9 +13592,9 @@
         <v>-0.96312533288099345</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -13621,9 +13621,9 @@
         <v>-1.5026790670657939</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -13650,9 +13650,9 @@
         <v>-1.8309231951944649</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -13679,9 +13679,9 @@
         <v>-2.0723760699848621</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -13708,9 +13708,9 @@
         <v>-2.2479372020534059</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -13737,9 +13737,9 @@
         <v>-2.3970612827093651</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -13766,9 +13766,9 @@
         <v>-2.519257662987366</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -13795,9 +13795,9 @@
         <v>-2.6277142063509982</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -13824,9 +13824,9 @@
         <v>-2.7226656488664198</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -13853,9 +13853,9 @@
         <v>-2.8070983677360348</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -13882,9 +13882,9 @@
         <v>-2.9931799380567221</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -13911,9 +13911,9 @@
         <v>-0.9078725854577725</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -13940,9 +13940,9 @@
         <v>-1.519802127747945</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -13969,9 +13969,9 @@
         <v>-1.8521920596270121</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -13998,9 +13998,9 @@
         <v>-2.094214575116697</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -14027,9 +14027,9 @@
         <v>-2.281769135464939</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -14056,9 +14056,9 @@
         <v>-2.4334401852763912</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -14085,9 +14085,9 @@
         <v>-2.5581156367701641</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -14114,9 +14114,9 @@
         <v>-2.6714669829785902</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -14143,9 +14143,9 @@
         <v>-2.7701993860012339</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -14172,9 +14172,9 @@
         <v>-2.8629353362818502</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>
@@ -14209,9 +14209,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A55AFA4-8F1B-A741-95DC-BBCE6D22B32F}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -14222,38 +14222,38 @@
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="I2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I2" s="29" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>65</v>
@@ -14280,9 +14280,9 @@
         <v>-0.63677377983195127</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>131</v>
@@ -14309,9 +14309,9 @@
         <v>-0.90505447920028792</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>196</v>
@@ -14338,9 +14338,9 @@
         <v>-1.055709693450388</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6">
         <v>262</v>
@@ -14367,9 +14367,9 @@
         <v>-1.1678881899628679</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
         <v>328</v>
@@ -14396,9 +14396,9 @@
         <v>-1.2531109174619821</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8">
         <v>393</v>
@@ -14425,9 +14425,9 @@
         <v>-1.3241851284082169</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>459</v>
@@ -14454,9 +14454,9 @@
         <v>-1.383808948259927</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>524</v>
@@ -14483,9 +14483,9 @@
         <v>-1.434215555257919</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>590</v>
@@ -14512,9 +14512,9 @@
         <v>-1.4806034372918011</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12">
         <v>656</v>
@@ -14541,9 +14541,9 @@
         <v>-1.5219065035189721</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>666</v>
@@ -14570,9 +14570,9 @@
         <v>-1.6087284980397041</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>65</v>
@@ -14599,9 +14599,9 @@
         <v>-0.66743378565601574</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>130</v>
@@ -14628,9 +14628,9 @@
         <v>-0.93011496123636617</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16">
         <v>196</v>
@@ -14657,9 +14657,9 @@
         <v>-1.0905624346294061</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17">
         <v>262</v>
@@ -14686,9 +14686,9 @@
         <v>-1.2001895398480109</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>327</v>
@@ -14715,9 +14715,9 @@
         <v>-1.2867004300291389</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>393</v>
@@ -14744,9 +14744,9 @@
         <v>-1.355086884184499</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20">
         <v>458</v>
@@ -14773,9 +14773,9 @@
         <v>-1.413717438137748</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>524</v>
@@ -14802,9 +14802,9 @@
         <v>-1.4665843339534821</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22">
         <v>589</v>
@@ -14831,9 +14831,9 @@
         <v>-1.510178228411488</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23">
         <v>655</v>
@@ -14860,9 +14860,9 @@
         <v>-1.549703163103892</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24">
         <v>665</v>
@@ -14889,9 +14889,9 @@
         <v>-1.6384192945088669</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25">
         <v>65</v>
@@ -14918,9 +14918,9 @@
         <v>-0.6476034812557715</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26">
         <v>130</v>
@@ -14947,9 +14947,9 @@
         <v>-0.90473833236534196</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>196</v>
@@ -14976,9 +14976,9 @@
         <v>-1.061169471038637</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>262</v>
@@ -15005,9 +15005,9 @@
         <v>-1.176238545860278</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29">
         <v>327</v>
@@ -15034,9 +15034,9 @@
         <v>-1.2599056260692181</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>393</v>
@@ -15063,9 +15063,9 @@
         <v>-1.33097361401347</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
         <v>458</v>
@@ -15092,9 +15092,9 @@
         <v>-1.389208681362945</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32">
         <v>524</v>
@@ -15121,9 +15121,9 @@
         <v>-1.440895761560437</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33">
         <v>589</v>
@@ -15150,9 +15150,9 @@
         <v>-1.486146722654665</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
         <v>655</v>
@@ -15179,9 +15179,9 @@
         <v>-1.5263847809235349</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>665</v>
@@ -15208,9 +15208,9 @@
         <v>-1.6150655810869099</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>65</v>
@@ -15237,9 +15237,9 @@
         <v>-0.59819379922267901</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37">
         <v>130</v>
@@ -15266,9 +15266,9 @@
         <v>-0.87468391726347172</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38">
         <v>196</v>
@@ -15295,9 +15295,9 @@
         <v>-1.024868742720443</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39">
         <v>262</v>
@@ -15324,9 +15324,9 @@
         <v>-1.134222564119282</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>327</v>
@@ -15353,9 +15353,9 @@
         <v>-1.2189659519539291</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B41">
         <v>393</v>
@@ -15382,9 +15382,9 @@
         <v>-1.287495976356402</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42">
         <v>458</v>
@@ -15411,9 +15411,9 @@
         <v>-1.3438284916510399</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43">
         <v>524</v>
@@ -15440,9 +15440,9 @@
         <v>-1.3950443995739641</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B44">
         <v>589</v>
@@ -15469,9 +15469,9 @@
         <v>-1.4396549827859071</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45">
         <v>655</v>
@@ -15498,9 +15498,9 @@
         <v>-1.4815561692260191</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46">
         <v>665</v>

</xml_diff>